<commit_message>
readme final polish, added relative paths, cleaned test folder
</commit_message>
<xml_diff>
--- a/outputs/reviews/openclaw_submission/openclaw_submission_review.xlsx
+++ b/outputs/reviews/openclaw_submission/openclaw_submission_review.xlsx
@@ -13303,7 +13303,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>e3f743f5-1e8a-4d2b-85f3-ee269a52ca26</t>
+          <t>c05aef74-85e2-4048-80c9-33744878a47f</t>
         </is>
       </c>
     </row>
@@ -13315,7 +13315,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-25T09:50:46+00:00</t>
+          <t>2026-05-25T10:27:51+00:00</t>
         </is>
       </c>
     </row>
@@ -13491,7 +13491,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>e3f743f5-1e8a-4d2b-85f3-ee269a52ca26</t>
+          <t>c05aef74-85e2-4048-80c9-33744878a47f</t>
         </is>
       </c>
     </row>
@@ -13527,7 +13527,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-25T09:50:46+00:00</t>
+          <t>2026-05-25T10:27:51+00:00</t>
         </is>
       </c>
     </row>
@@ -13619,7 +13619,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-25T09:50:46+00:00</t>
+          <t>2026-05-25T10:27:51+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>